<commit_message>
PPC: cierre semana 11 (PPC 29%), metas semana 12 (8 compromisos)
- Registra cierre de la semana 11 en index.json (entra a la grafica)
- Anade semana 12 (29 jun - 5 jul) con sus metas; queda como semana en curso
- Actas de cierre semanas 10 y 11

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/ppc/metas/semana-11.xlsx
+++ b/data/ppc/metas/semana-11.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e685dc9ab05c5d49/03. EZ PROJECT MANAGEMENT/06. CLAUDE CODE/15. PASADENA - TABLERO DE CONTROL/data/ppc/metas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="8_{9F6118ED-C808-49DE-8C8F-7E5F8323C680}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A25ABC46-8EE3-4BC6-9AAB-1B38F745C312}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="8_{9F6118ED-C808-49DE-8C8F-7E5F8323C680}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5DFEC2AA-1D77-49E2-82C2-59A7F454AD43}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Metas Semana 09" sheetId="1" r:id="rId1"/>
+    <sheet name="Metas Semana 11" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>

</xml_diff>